<commit_message>
añadiendo toda la estimacion del 2025
</commit_message>
<xml_diff>
--- a/Estimacion_error/datos_aves_marinas/2025/abril/Rompeolas/optimo_smape_por_clase.xlsx
+++ b/Estimacion_error/datos_aves_marinas/2025/abril/Rompeolas/optimo_smape_por_clase.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renzo\Desktop\Data_Saiensss\Estadística\Trabajos (laborales)\BMAP\Proyectos\conteo-aves-bmap\Estimacion_error\datos_aves_marinas\2025\abril\Rompeolas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02E74866-A015-49B5-AEAD-97603E5F9468}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF50A238-FA49-487C-B891-09958DF019C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="29">
   <si>
     <t>Clase</t>
   </si>
@@ -118,6 +118,9 @@
   </si>
   <si>
     <t>Con Balanceo + sahi:</t>
+  </si>
+  <si>
+    <t>Balanceo + sahi+ todas las fotos del RLOF</t>
   </si>
 </sst>
 </file>
@@ -266,6 +269,50 @@
         <a:xfrm>
           <a:off x="0" y="5562600"/>
           <a:ext cx="4952381" cy="1400000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>561375</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>123648</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Imagen 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{55CF3CE6-A3B1-4FEC-A34E-2FA40517CA5C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="28575" y="7467600"/>
+          <a:ext cx="4800000" cy="1419048"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -598,7 +645,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
@@ -875,6 +922,11 @@
         <v>27</v>
       </c>
     </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
añadiendo gifs a el flujo integrado de predicciones
</commit_message>
<xml_diff>
--- a/Estimacion_error/datos_aves_marinas/2025/abril/Rompeolas/optimo_smape_por_clase.xlsx
+++ b/Estimacion_error/datos_aves_marinas/2025/abril/Rompeolas/optimo_smape_por_clase.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renzo\Desktop\Data_Saiensss\Estadística\Trabajos (laborales)\BMAP\Proyectos\conteo-aves-bmap\Estimacion_error\datos_aves_marinas\2025\abril\Rompeolas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renzo\Desktop\Estadística\Trabajos (laborales)\BMAP\Proyectos\conteo-aves-bmap\Estimacion_error\datos_aves_marinas\2025\abril\Rompeolas\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF50A238-FA49-487C-B891-09958DF019C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,9 +25,6 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -325,9 +322,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -365,9 +362,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -400,26 +397,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -452,26 +432,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -646,13 +609,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -672,7 +635,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -692,7 +655,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -712,7 +675,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -732,7 +695,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -752,7 +715,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -772,7 +735,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>14</v>
       </c>
@@ -792,7 +755,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>16</v>
       </c>
@@ -812,7 +775,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>17</v>
       </c>
@@ -832,7 +795,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>19</v>
       </c>
@@ -852,7 +815,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>21</v>
       </c>
@@ -872,7 +835,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>22</v>
       </c>
@@ -892,7 +855,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -912,17 +875,17 @@
         <v>115</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>28</v>
       </c>

</xml_diff>